<commit_message>
Group B: paste group A's per-size FS end tables (identical values), FS6809-04 + bulkhead rows
- tools_fs: NWO_FS -04 / -24 and FSBH_MEAS -04 / -10 / -16 from claude/ecstatic-hopper-fk5p40 fsends_20261021/entries.json;
  FSM_SRC / FSBH_ASSUME / NWOFS_ASSUME take the group A wording (FSM / NWO_FS -06..-20 values already equal)
- regen 224 new, 0 lost (changed: AxialSource wording only); checks clean; FS forged closed loop 56 cfg / 1599 checks, 0 off
- 127 of 168 group B parts; README sections 1 / 8 list the configurations from the user's answers and STEPs

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Sbz7LkX6Jr9QuSxTU76dzT
</commit_message>
<xml_diff>
--- a/tools/_out/groupB_20261021/out/fs/DesignTable_FS2403_SW2.xlsx
+++ b/tools/_out/groupB_20261021/out/fs/DesignTable_FS2403_SW2.xlsx
@@ -960,7 +960,7 @@
       </c>
       <c r="AS3" t="inlineStr">
         <is>
-          <t>Air-Way FF2403 (s9, double-pass 2026-10-15, parts.air-way.com/api/series/9, two fetches identical) [user 2026-10-15: "use airway dimensions, check brennan too"]; checked against the Brennan ORFS catalog p3 FS2403-04-04 (ORFS-p003-t03) | MODEL: L6 face -&gt; face, hex S1, bores D1 (both sides): review table (Air-Way, staged FS table; OMi website list decides the parts); hex over the whole length between the two ends; bore step at the hex mid-plane (ASSUMPTION, as 2403; no effect where the two bores are equal); hex end chamfers NOT modelled; male O-ring face-seal end (SAE J1453): thread = the face-seal thread of the dash (Air-Way callout = Brennan ORFS catalog); face O-ring groove (inner / outer dia, depth), land, 45deg nose chamfer, thread length, 60deg flank, relief and end length measured on the Brennan pilot of that dash (Brennan FS2403-04-04 (both ends; fsmeasure.measure_fsm, group B 2026-10-21); single manufacturer - Air-Way 3D models not yet measured, Q-FS-2NDSHAPE); groove drawn rectangular (its outer bottom corner is hidden under the O-ring Brennan fuses into the solid - ASSUMPTION); O-ring not modelled (separate FS4000 part); male O-ring face-seal end (SAE J1453): thread = the face-seal thread of the dash (Air-Way callout = Brennan ORFS catalog); face O-ring groove (inner / outer dia, depth), land, 45deg nose chamfer, thread length, 60deg flank, relief and end length measured on the Brennan pilot of that dash (Brennan FS2403-04-04 (both ends; fsmeasure.measure_fsm, group B 2026-10-21); single manufacturer - Air-Way 3D models not yet measured, Q-FS-2NDSHAPE); groove drawn rectangular (its outer bottom corner is hidden under the O-ring Brennan fuses into the solid - ASSUMPTION); O-ring not modelled (separate FS4000 part)</t>
+          <t>Air-Way FF2403 (s9, double-pass 2026-10-15, parts.air-way.com/api/series/9, two fetches identical) [user 2026-10-15: "use airway dimensions, check brennan too"]; checked against the Brennan ORFS catalog p3 FS2403-04-04 (ORFS-p003-t03) | MODEL: L6 face -&gt; face, hex S1, bores D1 (both sides): review table (Air-Way, staged FS table; OMi website list decides the parts); hex over the whole length between the two ends; bore step at the hex mid-plane (ASSUMPTION, as 2403; no effect where the two bores are equal); hex end chamfers NOT modelled; male O-ring face-seal end (SAE J1453): thread = the face-seal thread of the dash (Air-Way callout = Brennan ORFS catalog); face O-ring groove (inner / outer dia, depth), land, 45deg nose chamfer, thread length, 60deg flank, relief and end length measured on the Brennan pilot of that dash (Brennan FS2403-04-04 (both ends; fsmeasure.measure_fsm, fsends_20261021); single manufacturer - Air-Way 3D models not yet measured, Q-FS-2NDSHAPE); groove drawn rectangular (its outer bottom corner is hidden under the O-ring Brennan fuses into the solid - ASSUMPTION); O-ring not modelled (separate FS4000 part); male O-ring face-seal end (SAE J1453): thread = the face-seal thread of the dash (Air-Way callout = Brennan ORFS catalog); face O-ring groove (inner / outer dia, depth), land, 45deg nose chamfer, thread length, 60deg flank, relief and end length measured on the Brennan pilot of that dash (Brennan FS2403-04-04 (both ends; fsmeasure.measure_fsm, fsends_20261021); single manufacturer - Air-Way 3D models not yet measured, Q-FS-2NDSHAPE); groove drawn rectangular (its outer bottom corner is hidden under the O-ring Brennan fuses into the solid - ASSUMPTION); O-ring not modelled (separate FS4000 part)</t>
         </is>
       </c>
       <c r="AT3" t="inlineStr">
@@ -1123,7 +1123,7 @@
       </c>
       <c r="AS4" t="inlineStr">
         <is>
-          <t>Air-Way FF2403 (s9, double-pass 2026-10-15, parts.air-way.com/api/series/9, two fetches identical) [user 2026-10-15: "use airway dimensions, check brennan too"]; checked against the Brennan ORFS catalog p3 FS2403-06-04 (ORFS-p003-t03) | MODEL: L6 face -&gt; face, hex S1, bores D1 (both sides): review table (Air-Way, staged FS table; OMi website list decides the parts); hex over the whole length between the two ends; bore step at the hex mid-plane (ASSUMPTION, as 2403; no effect where the two bores are equal); hex end chamfers NOT modelled; male O-ring face-seal end (SAE J1453): thread = the face-seal thread of the dash (Air-Way callout = Brennan ORFS catalog); face O-ring groove (inner / outer dia, depth), land, 45deg nose chamfer, thread length, 60deg flank, relief and end length measured on the Brennan pilot of that dash (Brennan FS2403-06-06 (both ends; fsmeasure.measure_fsm, group B 2026-10-21); single manufacturer - Air-Way 3D models not yet measured, Q-FS-2NDSHAPE); groove drawn rectangular (its outer bottom corner is hidden under the O-ring Brennan fuses into the solid - ASSUMPTION); O-ring not modelled (separate FS4000 part); male O-ring face-seal end (SAE J1453): thread = the face-seal thread of the dash (Air-Way callout = Brennan ORFS catalog); face O-ring groove (inner / outer dia, depth), land, 45deg nose chamfer, thread length, 60deg flank, relief and end length measured on the Brennan pilot of that dash (Brennan FS2403-04-04 (both ends; fsmeasure.measure_fsm, group B 2026-10-21); single manufacturer - Air-Way 3D models not yet measured, Q-FS-2NDSHAPE); groove drawn rectangular (its outer bottom corner is hidden under the O-ring Brennan fuses into the solid - ASSUMPTION); O-ring not modelled (separate FS4000 part)</t>
+          <t>Air-Way FF2403 (s9, double-pass 2026-10-15, parts.air-way.com/api/series/9, two fetches identical) [user 2026-10-15: "use airway dimensions, check brennan too"]; checked against the Brennan ORFS catalog p3 FS2403-06-04 (ORFS-p003-t03) | MODEL: L6 face -&gt; face, hex S1, bores D1 (both sides): review table (Air-Way, staged FS table; OMi website list decides the parts); hex over the whole length between the two ends; bore step at the hex mid-plane (ASSUMPTION, as 2403; no effect where the two bores are equal); hex end chamfers NOT modelled; male O-ring face-seal end (SAE J1453): thread = the face-seal thread of the dash (Air-Way callout = Brennan ORFS catalog); face O-ring groove (inner / outer dia, depth), land, 45deg nose chamfer, thread length, 60deg flank, relief and end length measured on the Brennan pilot of that dash (Brennan FS2403-06-06 (both ends; fsmeasure.measure_fsm, fsends_20261021); single manufacturer - Air-Way 3D models not yet measured, Q-FS-2NDSHAPE); groove drawn rectangular (its outer bottom corner is hidden under the O-ring Brennan fuses into the solid - ASSUMPTION); O-ring not modelled (separate FS4000 part); male O-ring face-seal end (SAE J1453): thread = the face-seal thread of the dash (Air-Way callout = Brennan ORFS catalog); face O-ring groove (inner / outer dia, depth), land, 45deg nose chamfer, thread length, 60deg flank, relief and end length measured on the Brennan pilot of that dash (Brennan FS2403-04-04 (both ends; fsmeasure.measure_fsm, fsends_20261021); single manufacturer - Air-Way 3D models not yet measured, Q-FS-2NDSHAPE); groove drawn rectangular (its outer bottom corner is hidden under the O-ring Brennan fuses into the solid - ASSUMPTION); O-ring not modelled (separate FS4000 part)</t>
         </is>
       </c>
       <c r="AT4" t="inlineStr">
@@ -1286,7 +1286,7 @@
       </c>
       <c r="AS5" t="inlineStr">
         <is>
-          <t>Air-Way FF2403 (s9, double-pass 2026-10-15, parts.air-way.com/api/series/9, two fetches identical) [user 2026-10-15: "use airway dimensions, check brennan too"]; checked against the Brennan ORFS catalog p3 FS2403-06-06 (ORFS-p003-t03) | MODEL: L6 face -&gt; face, hex S1, bores D1 (both sides): review table (Air-Way, staged FS table; OMi website list decides the parts); hex over the whole length between the two ends; bore step at the hex mid-plane (ASSUMPTION, as 2403; no effect where the two bores are equal); hex end chamfers NOT modelled; male O-ring face-seal end (SAE J1453): thread = the face-seal thread of the dash (Air-Way callout = Brennan ORFS catalog); face O-ring groove (inner / outer dia, depth), land, 45deg nose chamfer, thread length, 60deg flank, relief and end length measured on the Brennan pilot of that dash (Brennan FS2403-06-06 (both ends; fsmeasure.measure_fsm, group B 2026-10-21); single manufacturer - Air-Way 3D models not yet measured, Q-FS-2NDSHAPE); groove drawn rectangular (its outer bottom corner is hidden under the O-ring Brennan fuses into the solid - ASSUMPTION); O-ring not modelled (separate FS4000 part); male O-ring face-seal end (SAE J1453): thread = the face-seal thread of the dash (Air-Way callout = Brennan ORFS catalog); face O-ring groove (inner / outer dia, depth), land, 45deg nose chamfer, thread length, 60deg flank, relief and end length measured on the Brennan pilot of that dash (Brennan FS2403-06-06 (both ends; fsmeasure.measure_fsm, group B 2026-10-21); single manufacturer - Air-Way 3D models not yet measured, Q-FS-2NDSHAPE); groove drawn rectangular (its outer bottom corner is hidden under the O-ring Brennan fuses into the solid - ASSUMPTION); O-ring not modelled (separate FS4000 part)</t>
+          <t>Air-Way FF2403 (s9, double-pass 2026-10-15, parts.air-way.com/api/series/9, two fetches identical) [user 2026-10-15: "use airway dimensions, check brennan too"]; checked against the Brennan ORFS catalog p3 FS2403-06-06 (ORFS-p003-t03) | MODEL: L6 face -&gt; face, hex S1, bores D1 (both sides): review table (Air-Way, staged FS table; OMi website list decides the parts); hex over the whole length between the two ends; bore step at the hex mid-plane (ASSUMPTION, as 2403; no effect where the two bores are equal); hex end chamfers NOT modelled; male O-ring face-seal end (SAE J1453): thread = the face-seal thread of the dash (Air-Way callout = Brennan ORFS catalog); face O-ring groove (inner / outer dia, depth), land, 45deg nose chamfer, thread length, 60deg flank, relief and end length measured on the Brennan pilot of that dash (Brennan FS2403-06-06 (both ends; fsmeasure.measure_fsm, fsends_20261021); single manufacturer - Air-Way 3D models not yet measured, Q-FS-2NDSHAPE); groove drawn rectangular (its outer bottom corner is hidden under the O-ring Brennan fuses into the solid - ASSUMPTION); O-ring not modelled (separate FS4000 part); male O-ring face-seal end (SAE J1453): thread = the face-seal thread of the dash (Air-Way callout = Brennan ORFS catalog); face O-ring groove (inner / outer dia, depth), land, 45deg nose chamfer, thread length, 60deg flank, relief and end length measured on the Brennan pilot of that dash (Brennan FS2403-06-06 (both ends; fsmeasure.measure_fsm, fsends_20261021); single manufacturer - Air-Way 3D models not yet measured, Q-FS-2NDSHAPE); groove drawn rectangular (its outer bottom corner is hidden under the O-ring Brennan fuses into the solid - ASSUMPTION); O-ring not modelled (separate FS4000 part)</t>
         </is>
       </c>
       <c r="AT5" t="inlineStr">
@@ -1449,7 +1449,7 @@
       </c>
       <c r="AS6" t="inlineStr">
         <is>
-          <t>Air-Way FF2403 (s9, double-pass 2026-10-15, parts.air-way.com/api/series/9, two fetches identical) [user 2026-10-15: "use airway dimensions, check brennan too"]; checked against the Brennan ORFS catalog p3 FS2403-08-06 (ORFS-p003-t03) | MODEL: L6 face -&gt; face, hex S1, bores D1 (both sides): review table (Air-Way, staged FS table; OMi website list decides the parts); hex over the whole length between the two ends; bore step at the hex mid-plane (ASSUMPTION, as 2403; no effect where the two bores are equal); hex end chamfers NOT modelled; male O-ring face-seal end (SAE J1453): thread = the face-seal thread of the dash (Air-Way callout = Brennan ORFS catalog); face O-ring groove (inner / outer dia, depth), land, 45deg nose chamfer, thread length, 60deg flank, relief and end length measured on the Brennan pilot of that dash (Brennan FS2403-08-08 (both ends) = FS6400-08-08-O (fsmeasure.measure_fsm, orfs_wp2_20261020 checks (1)); single manufacturer - Air-Way 3D models not yet measured, Q-FS-2NDSHAPE); groove drawn rectangular (its outer bottom corner is hidden under the O-ring Brennan fuses into the solid - ASSUMPTION); O-ring not modelled (separate FS4000 part); male O-ring face-seal end (SAE J1453): thread = the face-seal thread of the dash (Air-Way callout = Brennan ORFS catalog); face O-ring groove (inner / outer dia, depth), land, 45deg nose chamfer, thread length, 60deg flank, relief and end length measured on the Brennan pilot of that dash (Brennan FS2403-06-06 (both ends; fsmeasure.measure_fsm, group B 2026-10-21); single manufacturer - Air-Way 3D models not yet measured, Q-FS-2NDSHAPE); groove drawn rectangular (its outer bottom corner is hidden under the O-ring Brennan fuses into the solid - ASSUMPTION); O-ring not modelled (separate FS4000 part)</t>
+          <t>Air-Way FF2403 (s9, double-pass 2026-10-15, parts.air-way.com/api/series/9, two fetches identical) [user 2026-10-15: "use airway dimensions, check brennan too"]; checked against the Brennan ORFS catalog p3 FS2403-08-06 (ORFS-p003-t03) | MODEL: L6 face -&gt; face, hex S1, bores D1 (both sides): review table (Air-Way, staged FS table; OMi website list decides the parts); hex over the whole length between the two ends; bore step at the hex mid-plane (ASSUMPTION, as 2403; no effect where the two bores are equal); hex end chamfers NOT modelled; male O-ring face-seal end (SAE J1453): thread = the face-seal thread of the dash (Air-Way callout = Brennan ORFS catalog); face O-ring groove (inner / outer dia, depth), land, 45deg nose chamfer, thread length, 60deg flank, relief and end length measured on the Brennan pilot of that dash (Brennan FS2403-08-08 (both ends) = FS6400-08-08-O (fsmeasure.measure_fsm, orfs_wp2_20261020 checks (1)); single manufacturer - Air-Way 3D models not yet measured, Q-FS-2NDSHAPE); groove drawn rectangular (its outer bottom corner is hidden under the O-ring Brennan fuses into the solid - ASSUMPTION); O-ring not modelled (separate FS4000 part); male O-ring face-seal end (SAE J1453): thread = the face-seal thread of the dash (Air-Way callout = Brennan ORFS catalog); face O-ring groove (inner / outer dia, depth), land, 45deg nose chamfer, thread length, 60deg flank, relief and end length measured on the Brennan pilot of that dash (Brennan FS2403-06-06 (both ends; fsmeasure.measure_fsm, fsends_20261021); single manufacturer - Air-Way 3D models not yet measured, Q-FS-2NDSHAPE); groove drawn rectangular (its outer bottom corner is hidden under the O-ring Brennan fuses into the solid - ASSUMPTION); O-ring not modelled (separate FS4000 part)</t>
         </is>
       </c>
       <c r="AT6" t="inlineStr">
@@ -1612,7 +1612,7 @@
       </c>
       <c r="AS7" t="inlineStr">
         <is>
-          <t>Air-Way FF2403 (s9, double-pass 2026-10-15, parts.air-way.com/api/series/9, two fetches identical) [user 2026-10-15: "use airway dimensions, check brennan too"]; checked against the Brennan ORFS catalog p3 FS2403-10-08 (ORFS-p003-t03) | MODEL: L6 face -&gt; face, hex S1, bores D1 (both sides): review table (Air-Way, staged FS table; OMi website list decides the parts); hex over the whole length between the two ends; bore step at the hex mid-plane (ASSUMPTION, as 2403; no effect where the two bores are equal); hex end chamfers NOT modelled; male O-ring face-seal end (SAE J1453): thread = the face-seal thread of the dash (Air-Way callout = Brennan ORFS catalog); face O-ring groove (inner / outer dia, depth), land, 45deg nose chamfer, thread length, 60deg flank, relief and end length measured on the Brennan pilot of that dash (Brennan FS2403-10-10 (both ends; fsmeasure.measure_fsm, group B 2026-10-21); single manufacturer - Air-Way 3D models not yet measured, Q-FS-2NDSHAPE); groove drawn rectangular (its outer bottom corner is hidden under the O-ring Brennan fuses into the solid - ASSUMPTION); O-ring not modelled (separate FS4000 part); male O-ring face-seal end (SAE J1453): thread = the face-seal thread of the dash (Air-Way callout = Brennan ORFS catalog); face O-ring groove (inner / outer dia, depth), land, 45deg nose chamfer, thread length, 60deg flank, relief and end length measured on the Brennan pilot of that dash (Brennan FS2403-08-08 (both ends) = FS6400-08-08-O (fsmeasure.measure_fsm, orfs_wp2_20261020 checks (1)); single manufacturer - Air-Way 3D models not yet measured, Q-FS-2NDSHAPE); groove drawn rectangular (its outer bottom corner is hidden under the O-ring Brennan fuses into the solid - ASSUMPTION); O-ring not modelled (separate FS4000 part)</t>
+          <t>Air-Way FF2403 (s9, double-pass 2026-10-15, parts.air-way.com/api/series/9, two fetches identical) [user 2026-10-15: "use airway dimensions, check brennan too"]; checked against the Brennan ORFS catalog p3 FS2403-10-08 (ORFS-p003-t03) | MODEL: L6 face -&gt; face, hex S1, bores D1 (both sides): review table (Air-Way, staged FS table; OMi website list decides the parts); hex over the whole length between the two ends; bore step at the hex mid-plane (ASSUMPTION, as 2403; no effect where the two bores are equal); hex end chamfers NOT modelled; male O-ring face-seal end (SAE J1453): thread = the face-seal thread of the dash (Air-Way callout = Brennan ORFS catalog); face O-ring groove (inner / outer dia, depth), land, 45deg nose chamfer, thread length, 60deg flank, relief and end length measured on the Brennan pilot of that dash (Brennan FS2403-10-10 (both ends; fsmeasure.measure_fsm, fsends_20261021); single manufacturer - Air-Way 3D models not yet measured, Q-FS-2NDSHAPE); groove drawn rectangular (its outer bottom corner is hidden under the O-ring Brennan fuses into the solid - ASSUMPTION); O-ring not modelled (separate FS4000 part); male O-ring face-seal end (SAE J1453): thread = the face-seal thread of the dash (Air-Way callout = Brennan ORFS catalog); face O-ring groove (inner / outer dia, depth), land, 45deg nose chamfer, thread length, 60deg flank, relief and end length measured on the Brennan pilot of that dash (Brennan FS2403-08-08 (both ends) = FS6400-08-08-O (fsmeasure.measure_fsm, orfs_wp2_20261020 checks (1)); single manufacturer - Air-Way 3D models not yet measured, Q-FS-2NDSHAPE); groove drawn rectangular (its outer bottom corner is hidden under the O-ring Brennan fuses into the solid - ASSUMPTION); O-ring not modelled (separate FS4000 part)</t>
         </is>
       </c>
       <c r="AT7" t="inlineStr">
@@ -1775,7 +1775,7 @@
       </c>
       <c r="AS8" t="inlineStr">
         <is>
-          <t>Air-Way FF2403 (s9, double-pass 2026-10-15, parts.air-way.com/api/series/9, two fetches identical) [user 2026-10-15: "use airway dimensions, check brennan too"]; checked against the Brennan ORFS catalog p3 FS2403-10-10 (ORFS-p003-t03) | MODEL: L6 face -&gt; face, hex S1, bores D1 (both sides): review table (Air-Way, staged FS table; OMi website list decides the parts); hex over the whole length between the two ends; bore step at the hex mid-plane (ASSUMPTION, as 2403; no effect where the two bores are equal); hex end chamfers NOT modelled; male O-ring face-seal end (SAE J1453): thread = the face-seal thread of the dash (Air-Way callout = Brennan ORFS catalog); face O-ring groove (inner / outer dia, depth), land, 45deg nose chamfer, thread length, 60deg flank, relief and end length measured on the Brennan pilot of that dash (Brennan FS2403-10-10 (both ends; fsmeasure.measure_fsm, group B 2026-10-21); single manufacturer - Air-Way 3D models not yet measured, Q-FS-2NDSHAPE); groove drawn rectangular (its outer bottom corner is hidden under the O-ring Brennan fuses into the solid - ASSUMPTION); O-ring not modelled (separate FS4000 part); male O-ring face-seal end (SAE J1453): thread = the face-seal thread of the dash (Air-Way callout = Brennan ORFS catalog); face O-ring groove (inner / outer dia, depth), land, 45deg nose chamfer, thread length, 60deg flank, relief and end length measured on the Brennan pilot of that dash (Brennan FS2403-10-10 (both ends; fsmeasure.measure_fsm, group B 2026-10-21); single manufacturer - Air-Way 3D models not yet measured, Q-FS-2NDSHAPE); groove drawn rectangular (its outer bottom corner is hidden under the O-ring Brennan fuses into the solid - ASSUMPTION); O-ring not modelled (separate FS4000 part)</t>
+          <t>Air-Way FF2403 (s9, double-pass 2026-10-15, parts.air-way.com/api/series/9, two fetches identical) [user 2026-10-15: "use airway dimensions, check brennan too"]; checked against the Brennan ORFS catalog p3 FS2403-10-10 (ORFS-p003-t03) | MODEL: L6 face -&gt; face, hex S1, bores D1 (both sides): review table (Air-Way, staged FS table; OMi website list decides the parts); hex over the whole length between the two ends; bore step at the hex mid-plane (ASSUMPTION, as 2403; no effect where the two bores are equal); hex end chamfers NOT modelled; male O-ring face-seal end (SAE J1453): thread = the face-seal thread of the dash (Air-Way callout = Brennan ORFS catalog); face O-ring groove (inner / outer dia, depth), land, 45deg nose chamfer, thread length, 60deg flank, relief and end length measured on the Brennan pilot of that dash (Brennan FS2403-10-10 (both ends; fsmeasure.measure_fsm, fsends_20261021); single manufacturer - Air-Way 3D models not yet measured, Q-FS-2NDSHAPE); groove drawn rectangular (its outer bottom corner is hidden under the O-ring Brennan fuses into the solid - ASSUMPTION); O-ring not modelled (separate FS4000 part); male O-ring face-seal end (SAE J1453): thread = the face-seal thread of the dash (Air-Way callout = Brennan ORFS catalog); face O-ring groove (inner / outer dia, depth), land, 45deg nose chamfer, thread length, 60deg flank, relief and end length measured on the Brennan pilot of that dash (Brennan FS2403-10-10 (both ends; fsmeasure.measure_fsm, fsends_20261021); single manufacturer - Air-Way 3D models not yet measured, Q-FS-2NDSHAPE); groove drawn rectangular (its outer bottom corner is hidden under the O-ring Brennan fuses into the solid - ASSUMPTION); O-ring not modelled (separate FS4000 part)</t>
         </is>
       </c>
       <c r="AT8" t="inlineStr">
@@ -1938,7 +1938,7 @@
       </c>
       <c r="AS9" t="inlineStr">
         <is>
-          <t>Air-Way FF2403 (s9, double-pass 2026-10-15, parts.air-way.com/api/series/9, two fetches identical) [user 2026-10-15: "use airway dimensions, check brennan too"]; checked against the Brennan ORFS catalog p3 FS2403-12-08 (ORFS-p003-t03) | MODEL: L6 face -&gt; face, hex S1, bores D1 (both sides): review table (Air-Way, staged FS table; OMi website list decides the parts); hex over the whole length between the two ends; bore step at the hex mid-plane (ASSUMPTION, as 2403; no effect where the two bores are equal); hex end chamfers NOT modelled; male O-ring face-seal end (SAE J1453): thread = the face-seal thread of the dash (Air-Way callout = Brennan ORFS catalog); face O-ring groove (inner / outer dia, depth), land, 45deg nose chamfer, thread length, 60deg flank, relief and end length measured on the Brennan pilot of that dash (Brennan FS2403-12-12 (both ends; fsmeasure.measure_fsm, group B 2026-10-21); single manufacturer - Air-Way 3D models not yet measured, Q-FS-2NDSHAPE); groove drawn rectangular (its outer bottom corner is hidden under the O-ring Brennan fuses into the solid - ASSUMPTION); O-ring not modelled (separate FS4000 part); male O-ring face-seal end (SAE J1453): thread = the face-seal thread of the dash (Air-Way callout = Brennan ORFS catalog); face O-ring groove (inner / outer dia, depth), land, 45deg nose chamfer, thread length, 60deg flank, relief and end length measured on the Brennan pilot of that dash (Brennan FS2403-08-08 (both ends) = FS6400-08-08-O (fsmeasure.measure_fsm, orfs_wp2_20261020 checks (1)); single manufacturer - Air-Way 3D models not yet measured, Q-FS-2NDSHAPE); groove drawn rectangular (its outer bottom corner is hidden under the O-ring Brennan fuses into the solid - ASSUMPTION); O-ring not modelled (separate FS4000 part)</t>
+          <t>Air-Way FF2403 (s9, double-pass 2026-10-15, parts.air-way.com/api/series/9, two fetches identical) [user 2026-10-15: "use airway dimensions, check brennan too"]; checked against the Brennan ORFS catalog p3 FS2403-12-08 (ORFS-p003-t03) | MODEL: L6 face -&gt; face, hex S1, bores D1 (both sides): review table (Air-Way, staged FS table; OMi website list decides the parts); hex over the whole length between the two ends; bore step at the hex mid-plane (ASSUMPTION, as 2403; no effect where the two bores are equal); hex end chamfers NOT modelled; male O-ring face-seal end (SAE J1453): thread = the face-seal thread of the dash (Air-Way callout = Brennan ORFS catalog); face O-ring groove (inner / outer dia, depth), land, 45deg nose chamfer, thread length, 60deg flank, relief and end length measured on the Brennan pilot of that dash (Brennan FS2403-12-12 (both ends; fsmeasure.measure_fsm, fsends_20261021); single manufacturer - Air-Way 3D models not yet measured, Q-FS-2NDSHAPE); groove drawn rectangular (its outer bottom corner is hidden under the O-ring Brennan fuses into the solid - ASSUMPTION); O-ring not modelled (separate FS4000 part); male O-ring face-seal end (SAE J1453): thread = the face-seal thread of the dash (Air-Way callout = Brennan ORFS catalog); face O-ring groove (inner / outer dia, depth), land, 45deg nose chamfer, thread length, 60deg flank, relief and end length measured on the Brennan pilot of that dash (Brennan FS2403-08-08 (both ends) = FS6400-08-08-O (fsmeasure.measure_fsm, orfs_wp2_20261020 checks (1)); single manufacturer - Air-Way 3D models not yet measured, Q-FS-2NDSHAPE); groove drawn rectangular (its outer bottom corner is hidden under the O-ring Brennan fuses into the solid - ASSUMPTION); O-ring not modelled (separate FS4000 part)</t>
         </is>
       </c>
       <c r="AT9" t="inlineStr">
@@ -2101,7 +2101,7 @@
       </c>
       <c r="AS10" t="inlineStr">
         <is>
-          <t>Air-Way FF2403 (s9, double-pass 2026-10-15, parts.air-way.com/api/series/9, two fetches identical) [user 2026-10-15: "use airway dimensions, check brennan too"]; checked against the Brennan ORFS catalog p3 FS2403-12-10 (ORFS-p003-t03) | MODEL: L6 face -&gt; face, hex S1, bores D1 (both sides): review table (Air-Way, staged FS table; OMi website list decides the parts); hex over the whole length between the two ends; bore step at the hex mid-plane (ASSUMPTION, as 2403; no effect where the two bores are equal); hex end chamfers NOT modelled; male O-ring face-seal end (SAE J1453): thread = the face-seal thread of the dash (Air-Way callout = Brennan ORFS catalog); face O-ring groove (inner / outer dia, depth), land, 45deg nose chamfer, thread length, 60deg flank, relief and end length measured on the Brennan pilot of that dash (Brennan FS2403-12-12 (both ends; fsmeasure.measure_fsm, group B 2026-10-21); single manufacturer - Air-Way 3D models not yet measured, Q-FS-2NDSHAPE); groove drawn rectangular (its outer bottom corner is hidden under the O-ring Brennan fuses into the solid - ASSUMPTION); O-ring not modelled (separate FS4000 part); male O-ring face-seal end (SAE J1453): thread = the face-seal thread of the dash (Air-Way callout = Brennan ORFS catalog); face O-ring groove (inner / outer dia, depth), land, 45deg nose chamfer, thread length, 60deg flank, relief and end length measured on the Brennan pilot of that dash (Brennan FS2403-10-10 (both ends; fsmeasure.measure_fsm, group B 2026-10-21); single manufacturer - Air-Way 3D models not yet measured, Q-FS-2NDSHAPE); groove drawn rectangular (its outer bottom corner is hidden under the O-ring Brennan fuses into the solid - ASSUMPTION); O-ring not modelled (separate FS4000 part)</t>
+          <t>Air-Way FF2403 (s9, double-pass 2026-10-15, parts.air-way.com/api/series/9, two fetches identical) [user 2026-10-15: "use airway dimensions, check brennan too"]; checked against the Brennan ORFS catalog p3 FS2403-12-10 (ORFS-p003-t03) | MODEL: L6 face -&gt; face, hex S1, bores D1 (both sides): review table (Air-Way, staged FS table; OMi website list decides the parts); hex over the whole length between the two ends; bore step at the hex mid-plane (ASSUMPTION, as 2403; no effect where the two bores are equal); hex end chamfers NOT modelled; male O-ring face-seal end (SAE J1453): thread = the face-seal thread of the dash (Air-Way callout = Brennan ORFS catalog); face O-ring groove (inner / outer dia, depth), land, 45deg nose chamfer, thread length, 60deg flank, relief and end length measured on the Brennan pilot of that dash (Brennan FS2403-12-12 (both ends; fsmeasure.measure_fsm, fsends_20261021); single manufacturer - Air-Way 3D models not yet measured, Q-FS-2NDSHAPE); groove drawn rectangular (its outer bottom corner is hidden under the O-ring Brennan fuses into the solid - ASSUMPTION); O-ring not modelled (separate FS4000 part); male O-ring face-seal end (SAE J1453): thread = the face-seal thread of the dash (Air-Way callout = Brennan ORFS catalog); face O-ring groove (inner / outer dia, depth), land, 45deg nose chamfer, thread length, 60deg flank, relief and end length measured on the Brennan pilot of that dash (Brennan FS2403-10-10 (both ends; fsmeasure.measure_fsm, fsends_20261021); single manufacturer - Air-Way 3D models not yet measured, Q-FS-2NDSHAPE); groove drawn rectangular (its outer bottom corner is hidden under the O-ring Brennan fuses into the solid - ASSUMPTION); O-ring not modelled (separate FS4000 part)</t>
         </is>
       </c>
       <c r="AT10" t="inlineStr">
@@ -2264,7 +2264,7 @@
       </c>
       <c r="AS11" t="inlineStr">
         <is>
-          <t>Air-Way FF2403 (s9, double-pass 2026-10-15, parts.air-way.com/api/series/9, two fetches identical) [user 2026-10-15: "use airway dimensions, check brennan too"]; checked against the Brennan ORFS catalog p3 FS2403-12-12 (ORFS-p003-t03) | MODEL: L6 face -&gt; face, hex S1, bores D1 (both sides): review table (Air-Way, staged FS table; OMi website list decides the parts); hex over the whole length between the two ends; bore step at the hex mid-plane (ASSUMPTION, as 2403; no effect where the two bores are equal); hex end chamfers NOT modelled; male O-ring face-seal end (SAE J1453): thread = the face-seal thread of the dash (Air-Way callout = Brennan ORFS catalog); face O-ring groove (inner / outer dia, depth), land, 45deg nose chamfer, thread length, 60deg flank, relief and end length measured on the Brennan pilot of that dash (Brennan FS2403-12-12 (both ends; fsmeasure.measure_fsm, group B 2026-10-21); single manufacturer - Air-Way 3D models not yet measured, Q-FS-2NDSHAPE); groove drawn rectangular (its outer bottom corner is hidden under the O-ring Brennan fuses into the solid - ASSUMPTION); O-ring not modelled (separate FS4000 part); male O-ring face-seal end (SAE J1453): thread = the face-seal thread of the dash (Air-Way callout = Brennan ORFS catalog); face O-ring groove (inner / outer dia, depth), land, 45deg nose chamfer, thread length, 60deg flank, relief and end length measured on the Brennan pilot of that dash (Brennan FS2403-12-12 (both ends; fsmeasure.measure_fsm, group B 2026-10-21); single manufacturer - Air-Way 3D models not yet measured, Q-FS-2NDSHAPE); groove drawn rectangular (its outer bottom corner is hidden under the O-ring Brennan fuses into the solid - ASSUMPTION); O-ring not modelled (separate FS4000 part)</t>
+          <t>Air-Way FF2403 (s9, double-pass 2026-10-15, parts.air-way.com/api/series/9, two fetches identical) [user 2026-10-15: "use airway dimensions, check brennan too"]; checked against the Brennan ORFS catalog p3 FS2403-12-12 (ORFS-p003-t03) | MODEL: L6 face -&gt; face, hex S1, bores D1 (both sides): review table (Air-Way, staged FS table; OMi website list decides the parts); hex over the whole length between the two ends; bore step at the hex mid-plane (ASSUMPTION, as 2403; no effect where the two bores are equal); hex end chamfers NOT modelled; male O-ring face-seal end (SAE J1453): thread = the face-seal thread of the dash (Air-Way callout = Brennan ORFS catalog); face O-ring groove (inner / outer dia, depth), land, 45deg nose chamfer, thread length, 60deg flank, relief and end length measured on the Brennan pilot of that dash (Brennan FS2403-12-12 (both ends; fsmeasure.measure_fsm, fsends_20261021); single manufacturer - Air-Way 3D models not yet measured, Q-FS-2NDSHAPE); groove drawn rectangular (its outer bottom corner is hidden under the O-ring Brennan fuses into the solid - ASSUMPTION); O-ring not modelled (separate FS4000 part); male O-ring face-seal end (SAE J1453): thread = the face-seal thread of the dash (Air-Way callout = Brennan ORFS catalog); face O-ring groove (inner / outer dia, depth), land, 45deg nose chamfer, thread length, 60deg flank, relief and end length measured on the Brennan pilot of that dash (Brennan FS2403-12-12 (both ends; fsmeasure.measure_fsm, fsends_20261021); single manufacturer - Air-Way 3D models not yet measured, Q-FS-2NDSHAPE); groove drawn rectangular (its outer bottom corner is hidden under the O-ring Brennan fuses into the solid - ASSUMPTION); O-ring not modelled (separate FS4000 part)</t>
         </is>
       </c>
       <c r="AT11" t="inlineStr">
@@ -2427,7 +2427,7 @@
       </c>
       <c r="AS12" t="inlineStr">
         <is>
-          <t>Air-Way FF2403 (s9, double-pass 2026-10-15, parts.air-way.com/api/series/9, two fetches identical) [user 2026-10-15: "use airway dimensions, check brennan too"]; checked against the Brennan ORFS catalog p3 FS2403-16-12 (ORFS-p003-t03) | MODEL: L6 face -&gt; face, hex S1, bores D1 (both sides): review table (Air-Way, staged FS table; OMi website list decides the parts); hex over the whole length between the two ends; bore step at the hex mid-plane (ASSUMPTION, as 2403; no effect where the two bores are equal); hex end chamfers NOT modelled; male O-ring face-seal end (SAE J1453): thread = the face-seal thread of the dash (Air-Way callout = Brennan ORFS catalog); face O-ring groove (inner / outer dia, depth), land, 45deg nose chamfer, thread length, 60deg flank, relief and end length measured on the Brennan pilot of that dash (Brennan FS2403-16-16 (both ends; fsmeasure.measure_fsm, group B 2026-10-21); single manufacturer - Air-Way 3D models not yet measured, Q-FS-2NDSHAPE); groove drawn rectangular (its outer bottom corner is hidden under the O-ring Brennan fuses into the solid - ASSUMPTION); O-ring not modelled (separate FS4000 part); male O-ring face-seal end (SAE J1453): thread = the face-seal thread of the dash (Air-Way callout = Brennan ORFS catalog); face O-ring groove (inner / outer dia, depth), land, 45deg nose chamfer, thread length, 60deg flank, relief and end length measured on the Brennan pilot of that dash (Brennan FS2403-12-12 (both ends; fsmeasure.measure_fsm, group B 2026-10-21); single manufacturer - Air-Way 3D models not yet measured, Q-FS-2NDSHAPE); groove drawn rectangular (its outer bottom corner is hidden under the O-ring Brennan fuses into the solid - ASSUMPTION); O-ring not modelled (separate FS4000 part)</t>
+          <t>Air-Way FF2403 (s9, double-pass 2026-10-15, parts.air-way.com/api/series/9, two fetches identical) [user 2026-10-15: "use airway dimensions, check brennan too"]; checked against the Brennan ORFS catalog p3 FS2403-16-12 (ORFS-p003-t03) | MODEL: L6 face -&gt; face, hex S1, bores D1 (both sides): review table (Air-Way, staged FS table; OMi website list decides the parts); hex over the whole length between the two ends; bore step at the hex mid-plane (ASSUMPTION, as 2403; no effect where the two bores are equal); hex end chamfers NOT modelled; male O-ring face-seal end (SAE J1453): thread = the face-seal thread of the dash (Air-Way callout = Brennan ORFS catalog); face O-ring groove (inner / outer dia, depth), land, 45deg nose chamfer, thread length, 60deg flank, relief and end length measured on the Brennan pilot of that dash (Brennan FS2403-16-16 (both ends; fsmeasure.measure_fsm, fsends_20261021); single manufacturer - Air-Way 3D models not yet measured, Q-FS-2NDSHAPE); groove drawn rectangular (its outer bottom corner is hidden under the O-ring Brennan fuses into the solid - ASSUMPTION); O-ring not modelled (separate FS4000 part); male O-ring face-seal end (SAE J1453): thread = the face-seal thread of the dash (Air-Way callout = Brennan ORFS catalog); face O-ring groove (inner / outer dia, depth), land, 45deg nose chamfer, thread length, 60deg flank, relief and end length measured on the Brennan pilot of that dash (Brennan FS2403-12-12 (both ends; fsmeasure.measure_fsm, fsends_20261021); single manufacturer - Air-Way 3D models not yet measured, Q-FS-2NDSHAPE); groove drawn rectangular (its outer bottom corner is hidden under the O-ring Brennan fuses into the solid - ASSUMPTION); O-ring not modelled (separate FS4000 part)</t>
         </is>
       </c>
       <c r="AT12" t="inlineStr">
@@ -2590,7 +2590,7 @@
       </c>
       <c r="AS13" t="inlineStr">
         <is>
-          <t>Air-Way FF2403 (s9, double-pass 2026-10-15, parts.air-way.com/api/series/9, two fetches identical) [user 2026-10-15: "use airway dimensions, check brennan too"]; checked against the Brennan ORFS catalog p3 FS2403-16-16 (ORFS-p003-t03) | MODEL: L6 face -&gt; face, hex S1, bores D1 (both sides): review table (Air-Way, staged FS table; OMi website list decides the parts); hex over the whole length between the two ends; bore step at the hex mid-plane (ASSUMPTION, as 2403; no effect where the two bores are equal); hex end chamfers NOT modelled; male O-ring face-seal end (SAE J1453): thread = the face-seal thread of the dash (Air-Way callout = Brennan ORFS catalog); face O-ring groove (inner / outer dia, depth), land, 45deg nose chamfer, thread length, 60deg flank, relief and end length measured on the Brennan pilot of that dash (Brennan FS2403-16-16 (both ends; fsmeasure.measure_fsm, group B 2026-10-21); single manufacturer - Air-Way 3D models not yet measured, Q-FS-2NDSHAPE); groove drawn rectangular (its outer bottom corner is hidden under the O-ring Brennan fuses into the solid - ASSUMPTION); O-ring not modelled (separate FS4000 part); male O-ring face-seal end (SAE J1453): thread = the face-seal thread of the dash (Air-Way callout = Brennan ORFS catalog); face O-ring groove (inner / outer dia, depth), land, 45deg nose chamfer, thread length, 60deg flank, relief and end length measured on the Brennan pilot of that dash (Brennan FS2403-16-16 (both ends; fsmeasure.measure_fsm, group B 2026-10-21); single manufacturer - Air-Way 3D models not yet measured, Q-FS-2NDSHAPE); groove drawn rectangular (its outer bottom corner is hidden under the O-ring Brennan fuses into the solid - ASSUMPTION); O-ring not modelled (separate FS4000 part)</t>
+          <t>Air-Way FF2403 (s9, double-pass 2026-10-15, parts.air-way.com/api/series/9, two fetches identical) [user 2026-10-15: "use airway dimensions, check brennan too"]; checked against the Brennan ORFS catalog p3 FS2403-16-16 (ORFS-p003-t03) | MODEL: L6 face -&gt; face, hex S1, bores D1 (both sides): review table (Air-Way, staged FS table; OMi website list decides the parts); hex over the whole length between the two ends; bore step at the hex mid-plane (ASSUMPTION, as 2403; no effect where the two bores are equal); hex end chamfers NOT modelled; male O-ring face-seal end (SAE J1453): thread = the face-seal thread of the dash (Air-Way callout = Brennan ORFS catalog); face O-ring groove (inner / outer dia, depth), land, 45deg nose chamfer, thread length, 60deg flank, relief and end length measured on the Brennan pilot of that dash (Brennan FS2403-16-16 (both ends; fsmeasure.measure_fsm, fsends_20261021); single manufacturer - Air-Way 3D models not yet measured, Q-FS-2NDSHAPE); groove drawn rectangular (its outer bottom corner is hidden under the O-ring Brennan fuses into the solid - ASSUMPTION); O-ring not modelled (separate FS4000 part); male O-ring face-seal end (SAE J1453): thread = the face-seal thread of the dash (Air-Way callout = Brennan ORFS catalog); face O-ring groove (inner / outer dia, depth), land, 45deg nose chamfer, thread length, 60deg flank, relief and end length measured on the Brennan pilot of that dash (Brennan FS2403-16-16 (both ends; fsmeasure.measure_fsm, fsends_20261021); single manufacturer - Air-Way 3D models not yet measured, Q-FS-2NDSHAPE); groove drawn rectangular (its outer bottom corner is hidden under the O-ring Brennan fuses into the solid - ASSUMPTION); O-ring not modelled (separate FS4000 part)</t>
         </is>
       </c>
       <c r="AT13" t="inlineStr">
@@ -2753,7 +2753,7 @@
       </c>
       <c r="AS14" t="inlineStr">
         <is>
-          <t>Air-Way FF2403 (s9, double-pass 2026-10-15, parts.air-way.com/api/series/9, two fetches identical) [user 2026-10-15: "use airway dimensions, check brennan too"]; checked against the Brennan ORFS catalog p3 FS2403-20-16 (ORFS-p003-t03) | MODEL: L6 face -&gt; face, hex S1, bores D1 (both sides): review table (Air-Way, staged FS table; OMi website list decides the parts); hex over the whole length between the two ends; bore step at the hex mid-plane (ASSUMPTION, as 2403; no effect where the two bores are equal); hex end chamfers NOT modelled; male O-ring face-seal end (SAE J1453): thread = the face-seal thread of the dash (Air-Way callout = Brennan ORFS catalog); face O-ring groove (inner / outer dia, depth), land, 45deg nose chamfer, thread length, 60deg flank, relief and end length measured on the Brennan pilot of that dash (Brennan FS2403-20-20 (both ends; fsmeasure.measure_fsm, group B 2026-10-21); single manufacturer - Air-Way 3D models not yet measured, Q-FS-2NDSHAPE); groove drawn rectangular (its outer bottom corner is hidden under the O-ring Brennan fuses into the solid - ASSUMPTION); O-ring not modelled (separate FS4000 part); male O-ring face-seal end (SAE J1453): thread = the face-seal thread of the dash (Air-Way callout = Brennan ORFS catalog); face O-ring groove (inner / outer dia, depth), land, 45deg nose chamfer, thread length, 60deg flank, relief and end length measured on the Brennan pilot of that dash (Brennan FS2403-16-16 (both ends; fsmeasure.measure_fsm, group B 2026-10-21); single manufacturer - Air-Way 3D models not yet measured, Q-FS-2NDSHAPE); groove drawn rectangular (its outer bottom corner is hidden under the O-ring Brennan fuses into the solid - ASSUMPTION); O-ring not modelled (separate FS4000 part)</t>
+          <t>Air-Way FF2403 (s9, double-pass 2026-10-15, parts.air-way.com/api/series/9, two fetches identical) [user 2026-10-15: "use airway dimensions, check brennan too"]; checked against the Brennan ORFS catalog p3 FS2403-20-16 (ORFS-p003-t03) | MODEL: L6 face -&gt; face, hex S1, bores D1 (both sides): review table (Air-Way, staged FS table; OMi website list decides the parts); hex over the whole length between the two ends; bore step at the hex mid-plane (ASSUMPTION, as 2403; no effect where the two bores are equal); hex end chamfers NOT modelled; male O-ring face-seal end (SAE J1453): thread = the face-seal thread of the dash (Air-Way callout = Brennan ORFS catalog); face O-ring groove (inner / outer dia, depth), land, 45deg nose chamfer, thread length, 60deg flank, relief and end length measured on the Brennan pilot of that dash (Brennan FS2403-20-20 (both ends; fsmeasure.measure_fsm, fsends_20261021); single manufacturer - Air-Way 3D models not yet measured, Q-FS-2NDSHAPE); groove drawn rectangular (its outer bottom corner is hidden under the O-ring Brennan fuses into the solid - ASSUMPTION); O-ring not modelled (separate FS4000 part); male O-ring face-seal end (SAE J1453): thread = the face-seal thread of the dash (Air-Way callout = Brennan ORFS catalog); face O-ring groove (inner / outer dia, depth), land, 45deg nose chamfer, thread length, 60deg flank, relief and end length measured on the Brennan pilot of that dash (Brennan FS2403-16-16 (both ends; fsmeasure.measure_fsm, fsends_20261021); single manufacturer - Air-Way 3D models not yet measured, Q-FS-2NDSHAPE); groove drawn rectangular (its outer bottom corner is hidden under the O-ring Brennan fuses into the solid - ASSUMPTION); O-ring not modelled (separate FS4000 part)</t>
         </is>
       </c>
       <c r="AT14" t="inlineStr">
@@ -2916,7 +2916,7 @@
       </c>
       <c r="AS15" t="inlineStr">
         <is>
-          <t>Air-Way FF2403 (s9, double-pass 2026-10-15, parts.air-way.com/api/series/9, two fetches identical) [user 2026-10-15: "use airway dimensions, check brennan too"]; checked against the Brennan ORFS catalog p3 FS2403-20-20 (ORFS-p003-t03) | MODEL: L6 face -&gt; face, hex S1, bores D1 (both sides): review table (Air-Way, staged FS table; OMi website list decides the parts); hex over the whole length between the two ends; bore step at the hex mid-plane (ASSUMPTION, as 2403; no effect where the two bores are equal); hex end chamfers NOT modelled; male O-ring face-seal end (SAE J1453): thread = the face-seal thread of the dash (Air-Way callout = Brennan ORFS catalog); face O-ring groove (inner / outer dia, depth), land, 45deg nose chamfer, thread length, 60deg flank, relief and end length measured on the Brennan pilot of that dash (Brennan FS2403-20-20 (both ends; fsmeasure.measure_fsm, group B 2026-10-21); single manufacturer - Air-Way 3D models not yet measured, Q-FS-2NDSHAPE); groove drawn rectangular (its outer bottom corner is hidden under the O-ring Brennan fuses into the solid - ASSUMPTION); O-ring not modelled (separate FS4000 part); male O-ring face-seal end (SAE J1453): thread = the face-seal thread of the dash (Air-Way callout = Brennan ORFS catalog); face O-ring groove (inner / outer dia, depth), land, 45deg nose chamfer, thread length, 60deg flank, relief and end length measured on the Brennan pilot of that dash (Brennan FS2403-20-20 (both ends; fsmeasure.measure_fsm, group B 2026-10-21); single manufacturer - Air-Way 3D models not yet measured, Q-FS-2NDSHAPE); groove drawn rectangular (its outer bottom corner is hidden under the O-ring Brennan fuses into the solid - ASSUMPTION); O-ring not modelled (separate FS4000 part)</t>
+          <t>Air-Way FF2403 (s9, double-pass 2026-10-15, parts.air-way.com/api/series/9, two fetches identical) [user 2026-10-15: "use airway dimensions, check brennan too"]; checked against the Brennan ORFS catalog p3 FS2403-20-20 (ORFS-p003-t03) | MODEL: L6 face -&gt; face, hex S1, bores D1 (both sides): review table (Air-Way, staged FS table; OMi website list decides the parts); hex over the whole length between the two ends; bore step at the hex mid-plane (ASSUMPTION, as 2403; no effect where the two bores are equal); hex end chamfers NOT modelled; male O-ring face-seal end (SAE J1453): thread = the face-seal thread of the dash (Air-Way callout = Brennan ORFS catalog); face O-ring groove (inner / outer dia, depth), land, 45deg nose chamfer, thread length, 60deg flank, relief and end length measured on the Brennan pilot of that dash (Brennan FS2403-20-20 (both ends; fsmeasure.measure_fsm, fsends_20261021); single manufacturer - Air-Way 3D models not yet measured, Q-FS-2NDSHAPE); groove drawn rectangular (its outer bottom corner is hidden under the O-ring Brennan fuses into the solid - ASSUMPTION); O-ring not modelled (separate FS4000 part); male O-ring face-seal end (SAE J1453): thread = the face-seal thread of the dash (Air-Way callout = Brennan ORFS catalog); face O-ring groove (inner / outer dia, depth), land, 45deg nose chamfer, thread length, 60deg flank, relief and end length measured on the Brennan pilot of that dash (Brennan FS2403-20-20 (both ends; fsmeasure.measure_fsm, fsends_20261021); single manufacturer - Air-Way 3D models not yet measured, Q-FS-2NDSHAPE); groove drawn rectangular (its outer bottom corner is hidden under the O-ring Brennan fuses into the solid - ASSUMPTION); O-ring not modelled (separate FS4000 part)</t>
         </is>
       </c>
       <c r="AT15" t="inlineStr">
@@ -3079,7 +3079,7 @@
       </c>
       <c r="AS16" t="inlineStr">
         <is>
-          <t>[BRENNAN-ONLY 2026-10-18] no Air-Way row (FF2403 has no row of this size) -&gt; 2026-10-18 Brennan allowed (user: "yes use brennan but still differentiate"): L6@DRIVE: Brennan ORFS catalog p3 table ORFS-p003-t03 "FS2403 MFS-MFS STRAIGHT" row FS2403-24-20 col "FF LGTH" = "2.090" (07_RAW_EXTRACTS/brennan_catalogs/ORFS Catalog.pdf; tools/_out/brennan_catalog_20261001/catalog_verified.json, line_y 340.0, page verified True) [Brennan = yes 2026-10-18] - overall face -&gt; face; mapping: same-table check: 15/15 rows with an Air-Way value agree to rounding; S1HEX@HEX: Brennan ORFS catalog p3 table ORFS-p003-t03 "FS2403 MFS-MFS STRAIGHT" row FS2403-24-20 col "H HEX" = "2.125" (07_RAW_EXTRACTS/brennan_catalogs/ORFS Catalog.pdf; tools/_out/brennan_catalog_20261001/catalog_verified.json, line_y 340.0, page verified True) [Brennan = yes 2026-10-18] - body hex; mapping: same-table check: 15/15 rows with an Air-Way value agree to rounding; THDMAJ_D_1@DRIVE: end library: face-seal (SAE J1453) thread FS_THR of dash -24 = 2.0 (PLAN.md s2 FS_THR / the -24 thread of every staged ORFS row); = Brennan "A1 THREAD" "2-12" of this row [Q-TRANSFER-ENDLIB yes 2026-10-08]; THDMAJ_D_2@DRIVE: end library: face-seal (SAE J1453) thread FS_THR of dash -20 = 1.6875 (PLAN.md s2 FS_THR / the -20 thread of every staged ORFS row); = Brennan "A2 THREAD" "1-11/16-12" of this row [Q-TRANSFER-ENDLIB yes 2026-10-08]; $PRP@Thread_D_1: Brennan ORFS catalog p3 table ORFS-p003-t03 "FS2403 MFS-MFS STRAIGHT" row FS2403-24-20 col "A1 THREAD" "2-12" in the table's format; $PRP@Thread_D_2: Brennan ORFS catalog p3 table ORFS-p003-t03 "FS2403 MFS-MFS STRAIGHT" row FS2403-24-20 col "A2 THREAD" "1-11/16-12" in the table's format; D1_1@BORE: per-dash transfer, user 2026-10-18 Q-FS-XFER yes: same table FS2403: FSM -24 bore on 2 Air-Way row(s): 1.26 (unanimous) [Air-Way, not Brennan]; D1_2@BORE: per-dash transfer, user 2026-10-18 Q-FS-XFER yes: same table FS2403: FSM -20 bore on 3 Air-Way row(s): 1.02 (unanimous) [Air-Way, not Brennan] | MODEL: L6 face -&gt; face, hex S1, bores D1 (both sides): review table (Air-Way, staged FS table; OMi website list decides the parts); hex over the whole length between the two ends; bore step at the hex mid-plane (ASSUMPTION, as 2403; no effect where the two bores are equal); hex end chamfers NOT modelled; male O-ring face-seal end (SAE J1453): thread = the face-seal thread of the dash (Air-Way callout = Brennan ORFS catalog); face O-ring groove (inner / outer dia, depth), land, 45deg nose chamfer, thread length, 60deg flank, relief and end length measured on the Brennan pilot of that dash (Brennan FS2403-24-24 (both ends; fsmeasure.measure_fsm, orfs_steps2_20261020 ends_survey); single manufacturer - Air-Way 3D models not yet measured, Q-FS-2NDSHAPE); groove drawn rectangular (its outer bottom corner is hidden under the O-ring Brennan fuses into the solid - ASSUMPTION); O-ring not modelled (separate FS4000 part); male O-ring face-seal end (SAE J1453): thread = the face-seal thread of the dash (Air-Way callout = Brennan ORFS catalog); face O-ring groove (inner / outer dia, depth), land, 45deg nose chamfer, thread length, 60deg flank, relief and end length measured on the Brennan pilot of that dash (Brennan FS2403-20-20 (both ends; fsmeasure.measure_fsm, group B 2026-10-21); single manufacturer - Air-Way 3D models not yet measured, Q-FS-2NDSHAPE); groove drawn rectangular (its outer bottom corner is hidden under the O-ring Brennan fuses into the solid - ASSUMPTION); O-ring not modelled (separate FS4000 part)</t>
+          <t>[BRENNAN-ONLY 2026-10-18] no Air-Way row (FF2403 has no row of this size) -&gt; 2026-10-18 Brennan allowed (user: "yes use brennan but still differentiate"): L6@DRIVE: Brennan ORFS catalog p3 table ORFS-p003-t03 "FS2403 MFS-MFS STRAIGHT" row FS2403-24-20 col "FF LGTH" = "2.090" (07_RAW_EXTRACTS/brennan_catalogs/ORFS Catalog.pdf; tools/_out/brennan_catalog_20261001/catalog_verified.json, line_y 340.0, page verified True) [Brennan = yes 2026-10-18] - overall face -&gt; face; mapping: same-table check: 15/15 rows with an Air-Way value agree to rounding; S1HEX@HEX: Brennan ORFS catalog p3 table ORFS-p003-t03 "FS2403 MFS-MFS STRAIGHT" row FS2403-24-20 col "H HEX" = "2.125" (07_RAW_EXTRACTS/brennan_catalogs/ORFS Catalog.pdf; tools/_out/brennan_catalog_20261001/catalog_verified.json, line_y 340.0, page verified True) [Brennan = yes 2026-10-18] - body hex; mapping: same-table check: 15/15 rows with an Air-Way value agree to rounding; THDMAJ_D_1@DRIVE: end library: face-seal (SAE J1453) thread FS_THR of dash -24 = 2.0 (PLAN.md s2 FS_THR / the -24 thread of every staged ORFS row); = Brennan "A1 THREAD" "2-12" of this row [Q-TRANSFER-ENDLIB yes 2026-10-08]; THDMAJ_D_2@DRIVE: end library: face-seal (SAE J1453) thread FS_THR of dash -20 = 1.6875 (PLAN.md s2 FS_THR / the -20 thread of every staged ORFS row); = Brennan "A2 THREAD" "1-11/16-12" of this row [Q-TRANSFER-ENDLIB yes 2026-10-08]; $PRP@Thread_D_1: Brennan ORFS catalog p3 table ORFS-p003-t03 "FS2403 MFS-MFS STRAIGHT" row FS2403-24-20 col "A1 THREAD" "2-12" in the table's format; $PRP@Thread_D_2: Brennan ORFS catalog p3 table ORFS-p003-t03 "FS2403 MFS-MFS STRAIGHT" row FS2403-24-20 col "A2 THREAD" "1-11/16-12" in the table's format; D1_1@BORE: per-dash transfer, user 2026-10-18 Q-FS-XFER yes: same table FS2403: FSM -24 bore on 2 Air-Way row(s): 1.26 (unanimous) [Air-Way, not Brennan]; D1_2@BORE: per-dash transfer, user 2026-10-18 Q-FS-XFER yes: same table FS2403: FSM -20 bore on 3 Air-Way row(s): 1.02 (unanimous) [Air-Way, not Brennan] | MODEL: L6 face -&gt; face, hex S1, bores D1 (both sides): review table (Air-Way, staged FS table; OMi website list decides the parts); hex over the whole length between the two ends; bore step at the hex mid-plane (ASSUMPTION, as 2403; no effect where the two bores are equal); hex end chamfers NOT modelled; male O-ring face-seal end (SAE J1453): thread = the face-seal thread of the dash (Air-Way callout = Brennan ORFS catalog); face O-ring groove (inner / outer dia, depth), land, 45deg nose chamfer, thread length, 60deg flank, relief and end length measured on the Brennan pilot of that dash (Brennan FS2403-24-24 (both ends; fsmeasure.measure_fsm, orfs_steps2_20261020 ends_survey); single manufacturer - Air-Way 3D models not yet measured, Q-FS-2NDSHAPE); groove drawn rectangular (its outer bottom corner is hidden under the O-ring Brennan fuses into the solid - ASSUMPTION); O-ring not modelled (separate FS4000 part); male O-ring face-seal end (SAE J1453): thread = the face-seal thread of the dash (Air-Way callout = Brennan ORFS catalog); face O-ring groove (inner / outer dia, depth), land, 45deg nose chamfer, thread length, 60deg flank, relief and end length measured on the Brennan pilot of that dash (Brennan FS2403-20-20 (both ends; fsmeasure.measure_fsm, fsends_20261021); single manufacturer - Air-Way 3D models not yet measured, Q-FS-2NDSHAPE); groove drawn rectangular (its outer bottom corner is hidden under the O-ring Brennan fuses into the solid - ASSUMPTION); O-ring not modelled (separate FS4000 part)</t>
         </is>
       </c>
       <c r="AT16" t="inlineStr">

</xml_diff>